<commit_message>
Included fleece data to Thomas2007 test set
</commit_message>
<xml_diff>
--- a/Tests/Validation/Stock/Thomas2007Observed.xlsx
+++ b/Tests/Validation/Stock/Thomas2007Observed.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Repos\ApsimX\Tests\Validation\Stock\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KEO027\ApsimX\Tests\Validation\Stock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D13D98B1-C059-4B6D-BDA9-B43445D8E04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61FEA6B5-4482-4C4A-B4DF-601D2498AB2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ValidationData" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="23">
   <si>
     <t>SimulationName</t>
   </si>
@@ -104,6 +104,9 @@
   </si>
   <si>
     <t>OMD76</t>
+  </si>
+  <si>
+    <t>Stock.CFleeceWtAll</t>
   </si>
 </sst>
 </file>
@@ -446,21 +449,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1048564"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J1048564"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.81640625" customWidth="1"/>
-    <col min="3" max="3" width="10.1796875" customWidth="1"/>
-    <col min="4" max="4" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -488,8 +491,11 @@
       <c r="I1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f t="shared" ref="A2:A33" si="0">"Thomas2007"&amp;C2</f>
         <v>Thomas2007OMD55</v>
@@ -506,7 +512,7 @@
       </c>
       <c r="G2" s="3"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -524,7 +530,7 @@
       </c>
       <c r="G3" s="3"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -542,7 +548,7 @@
       </c>
       <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -560,7 +566,7 @@
       </c>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -584,7 +590,7 @@
         <v>1.7010000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -606,7 +612,7 @@
         <v>3.3620000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -628,7 +634,7 @@
         <v>5.1150000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -650,7 +656,7 @@
         <v>6.7700000000000005</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -672,7 +678,7 @@
         <v>8.4740000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -694,7 +700,7 @@
         <v>10.003</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -716,7 +722,7 @@
         <v>11.731999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -740,7 +746,7 @@
         <v>13.447999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -762,7 +768,7 @@
         <v>14.996999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -784,7 +790,7 @@
         <v>16.843999999999998</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -806,7 +812,7 @@
         <v>18.415999999999997</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -828,7 +834,7 @@
         <v>19.786999999999995</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -850,7 +856,7 @@
         <v>21.317999999999994</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -872,7 +878,7 @@
         <v>22.856999999999996</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -895,8 +901,11 @@
         <f t="shared" si="2"/>
         <v>24.999999999999996</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J20">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -918,7 +927,7 @@
         <v>26.737999999999996</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -940,7 +949,7 @@
         <v>28.357999999999997</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -962,7 +971,7 @@
         <v>30.159999999999997</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -984,7 +993,7 @@
         <v>31.869999999999997</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1006,7 +1015,7 @@
         <v>33.461999999999996</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1028,7 +1037,7 @@
         <v>34.858999999999995</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1052,7 +1061,7 @@
         <v>36.191999999999993</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1074,7 +1083,7 @@
         <v>37.620999999999995</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1096,7 +1105,7 @@
         <v>39.280999999999992</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1118,7 +1127,7 @@
         <v>40.699999999999989</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1140,7 +1149,7 @@
         <v>42.370999999999988</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1162,7 +1171,7 @@
         <v>44.023999999999987</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1184,7 +1193,7 @@
         <v>45.734999999999985</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="str">
         <f t="shared" ref="A34:A65" si="3">"Thomas2007"&amp;C34</f>
         <v>Thomas2007OMD55</v>
@@ -1208,7 +1217,7 @@
         <v>47.414999999999985</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1230,7 +1239,7 @@
         <v>49.031999999999982</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1252,7 +1261,7 @@
         <v>50.547999999999981</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1274,7 +1283,7 @@
         <v>52.21899999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1296,7 +1305,7 @@
         <v>53.830999999999982</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1318,7 +1327,7 @@
         <v>55.362999999999985</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1340,7 +1349,7 @@
         <v>57.091999999999985</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1365,7 +1374,7 @@
       </c>
       <c r="I41" s="2"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1388,7 +1397,7 @@
       </c>
       <c r="I42" s="2"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1411,7 +1420,7 @@
       </c>
       <c r="I43" s="2"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1434,7 +1443,7 @@
       </c>
       <c r="I44" s="2"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1457,7 +1466,7 @@
       </c>
       <c r="I45" s="2"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1480,7 +1489,7 @@
       </c>
       <c r="I46" s="2"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1503,7 +1512,7 @@
       </c>
       <c r="I47" s="2"/>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1527,8 +1536,11 @@
         <v>67.006999999999991</v>
       </c>
       <c r="I48" s="2"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J48">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1545,7 +1557,7 @@
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1562,7 +1574,7 @@
       </c>
       <c r="G50" s="3"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1579,7 +1591,7 @@
       </c>
       <c r="G51" s="3"/>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1596,7 +1608,7 @@
       </c>
       <c r="G52" s="3"/>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1619,7 +1631,7 @@
         <v>1.8580000000000001</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1640,7 +1652,7 @@
         <v>3.6230000000000002</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1661,7 +1673,7 @@
         <v>5.5760000000000005</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1682,7 +1694,7 @@
         <v>7.4970000000000008</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1703,7 +1715,7 @@
         <v>9.2580000000000009</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1724,7 +1736,7 @@
         <v>11.152000000000001</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1745,7 +1757,7 @@
         <v>13.008000000000001</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1768,7 +1780,7 @@
         <v>14.727</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1789,7 +1801,7 @@
         <v>16.615000000000002</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1810,7 +1822,7 @@
         <v>18.522000000000002</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1831,7 +1843,7 @@
         <v>20.412000000000003</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1852,7 +1864,7 @@
         <v>21.922000000000004</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1873,7 +1885,7 @@
         <v>23.846000000000004</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="str">
         <f t="shared" ref="A66:A97" si="6">"Thomas2007"&amp;C66</f>
         <v>Thomas2007OMD62</v>
@@ -1894,7 +1906,7 @@
         <v>25.546000000000003</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -1916,8 +1928,11 @@
         <f t="shared" si="4"/>
         <v>27.470000000000002</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J67">
+        <v>1.0589999999999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -1938,7 +1953,7 @@
         <v>29.201000000000004</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -1959,7 +1974,7 @@
         <v>31.190000000000005</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -1980,7 +1995,7 @@
         <v>33.086000000000006</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2001,7 +2016,7 @@
         <v>34.831000000000003</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2022,7 +2037,7 @@
         <v>36.690000000000005</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2043,7 +2058,7 @@
         <v>38.639000000000003</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2066,7 +2081,7 @@
         <v>40.504000000000005</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2087,7 +2102,7 @@
         <v>42.424000000000007</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2108,7 +2123,7 @@
         <v>44.27000000000001</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2129,7 +2144,7 @@
         <v>46.060000000000009</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2150,7 +2165,7 @@
         <v>47.808000000000007</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2171,7 +2186,7 @@
         <v>49.615000000000009</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2192,7 +2207,7 @@
         <v>51.484000000000009</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2215,7 +2230,7 @@
         <v>53.180000000000007</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2236,7 +2251,7 @@
         <v>55.225000000000009</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2257,7 +2272,7 @@
         <v>57.01100000000001</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2278,7 +2293,7 @@
         <v>58.876000000000012</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2299,7 +2314,7 @@
         <v>60.646000000000015</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2320,7 +2335,7 @@
         <v>62.418000000000013</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2341,7 +2356,7 @@
         <v>64.198000000000008</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2364,7 +2379,7 @@
         <v>65.494000000000014</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2385,7 +2400,7 @@
         <v>66.864000000000019</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2406,7 +2421,7 @@
         <v>67.793000000000021</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2427,7 +2442,7 @@
         <v>68.871000000000024</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2448,7 +2463,7 @@
         <v>70.183000000000021</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2469,7 +2484,7 @@
         <v>71.424000000000021</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2490,7 +2505,7 @@
         <v>72.673000000000016</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2512,8 +2527,11 @@
         <f t="shared" si="4"/>
         <v>73.836000000000013</v>
       </c>
-    </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J95">
+        <v>1.645</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD69</v>
@@ -2529,7 +2547,7 @@
       </c>
       <c r="G96" s="4"/>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD69</v>
@@ -2546,7 +2564,7 @@
       </c>
       <c r="G97" s="3"/>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" t="str">
         <f t="shared" ref="A98:A129" si="7">"Thomas2007"&amp;C98</f>
         <v>Thomas2007OMD69</v>
@@ -2563,7 +2581,7 @@
       </c>
       <c r="G98" s="3"/>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2580,7 +2598,7 @@
       </c>
       <c r="G99" s="3"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2603,7 +2621,7 @@
         <v>1.9810000000000001</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2624,7 +2642,7 @@
         <v>3.835</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2645,7 +2663,7 @@
         <v>5.4450000000000003</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2666,7 +2684,7 @@
         <v>7.3559999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2687,7 +2705,7 @@
         <v>9.0960000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2708,7 +2726,7 @@
         <v>10.975999999999999</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2729,7 +2747,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2752,7 +2770,7 @@
         <v>14.859</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2773,7 +2791,7 @@
         <v>16.728999999999999</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2794,7 +2812,7 @@
         <v>18.587</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2815,7 +2833,7 @@
         <v>20.402000000000001</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2836,7 +2854,7 @@
         <v>22.01</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2857,7 +2875,7 @@
         <v>23.807000000000002</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2878,7 +2896,7 @@
         <v>25.348000000000003</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2900,8 +2918,11 @@
         <f t="shared" si="8"/>
         <v>26.927000000000003</v>
       </c>
-    </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J114">
+        <v>1.286</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2922,7 +2943,7 @@
         <v>28.460000000000004</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2943,7 +2964,7 @@
         <v>29.873000000000005</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2964,7 +2985,7 @@
         <v>31.358000000000004</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2985,7 +3006,7 @@
         <v>32.867000000000004</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3006,7 +3027,7 @@
         <v>34.407000000000004</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3027,7 +3048,7 @@
         <v>36.185000000000002</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3050,7 +3071,7 @@
         <v>37.836000000000006</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A122" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3071,7 +3092,7 @@
         <v>39.587000000000003</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3092,7 +3113,7 @@
         <v>41.578000000000003</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3113,7 +3134,7 @@
         <v>43.268000000000001</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A125" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3134,7 +3155,7 @@
         <v>45.395000000000003</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A126" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3155,7 +3176,7 @@
         <v>47.103000000000002</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A127" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3176,7 +3197,7 @@
         <v>48.753</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3199,7 +3220,7 @@
         <v>50.494</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3220,7 +3241,7 @@
         <v>52.392000000000003</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A130" t="str">
         <f t="shared" ref="A130:A161" si="10">"Thomas2007"&amp;C130</f>
         <v>Thomas2007OMD69</v>
@@ -3241,7 +3262,7 @@
         <v>54.086000000000006</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A131" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3262,7 +3283,7 @@
         <v>55.818000000000005</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3283,7 +3304,7 @@
         <v>57.465000000000003</v>
       </c>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A133" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3304,7 +3325,7 @@
         <v>59.209000000000003</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A134" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3325,7 +3346,7 @@
         <v>61.029000000000003</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A135" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3348,7 +3369,7 @@
         <v>62.114000000000004</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A136" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3369,7 +3390,7 @@
         <v>63.574000000000005</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A137" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3390,7 +3411,7 @@
         <v>64.690000000000012</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A138" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3411,7 +3432,7 @@
         <v>65.849000000000018</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3432,7 +3453,7 @@
         <v>66.982000000000014</v>
       </c>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A140" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3453,7 +3474,7 @@
         <v>68.26700000000001</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A141" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3474,7 +3495,7 @@
         <v>69.572000000000017</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A142" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3496,8 +3517,11 @@
         <f t="shared" si="8"/>
         <v>70.968000000000018</v>
       </c>
-    </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J142">
+        <v>1.978</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A143" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3513,7 +3537,7 @@
       </c>
       <c r="G143" s="4"/>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A144" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3530,7 +3554,7 @@
       </c>
       <c r="G144" s="3"/>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A145" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3547,7 +3571,7 @@
       </c>
       <c r="G145" s="3"/>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A146" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3564,7 +3588,7 @@
       </c>
       <c r="G146" s="3"/>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A147" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3587,7 +3611,7 @@
         <v>1.9710000000000001</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A148" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3608,7 +3632,7 @@
         <v>3.415</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A149" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3629,7 +3653,7 @@
         <v>5.2989999999999995</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A150" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3650,7 +3674,7 @@
         <v>7.1389999999999993</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A151" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3671,7 +3695,7 @@
         <v>9.01</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3692,7 +3716,7 @@
         <v>10.725999999999999</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3713,7 +3737,7 @@
         <v>12.569999999999999</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3736,7 +3760,7 @@
         <v>14.206999999999999</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3757,7 +3781,7 @@
         <v>15.938999999999998</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3778,7 +3802,7 @@
         <v>17.680999999999997</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3799,7 +3823,7 @@
         <v>19.462999999999997</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3820,7 +3844,7 @@
         <v>20.680999999999997</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3841,7 +3865,7 @@
         <v>22.324999999999996</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3862,7 +3886,7 @@
         <v>23.977999999999994</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A161" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3884,8 +3908,11 @@
         <f t="shared" si="11"/>
         <v>25.483999999999995</v>
       </c>
-    </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J161">
+        <v>1.28</v>
+      </c>
+    </row>
+    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A162" t="str">
         <f t="shared" ref="A162:A182" si="12">"Thomas2007"&amp;C162</f>
         <v>Thomas2007OMD76</v>
@@ -3906,7 +3933,7 @@
         <v>26.875999999999994</v>
       </c>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A163" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -3927,7 +3954,7 @@
         <v>28.519999999999992</v>
       </c>
     </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A164" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -3948,7 +3975,7 @@
         <v>30.175999999999991</v>
       </c>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A165" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -3969,7 +3996,7 @@
         <v>31.570999999999991</v>
       </c>
     </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A166" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -3990,7 +4017,7 @@
         <v>33.142999999999994</v>
       </c>
     </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A167" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4011,7 +4038,7 @@
         <v>34.849999999999994</v>
       </c>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A168" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4034,7 +4061,7 @@
         <v>36.425999999999995</v>
       </c>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A169" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4055,7 +4082,7 @@
         <v>37.970999999999997</v>
       </c>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A170" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4076,7 +4103,7 @@
         <v>39.464999999999996</v>
       </c>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A171" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4097,7 +4124,7 @@
         <v>41.062999999999995</v>
       </c>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A172" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4118,7 +4145,7 @@
         <v>42.670999999999992</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A173" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4139,7 +4166,7 @@
         <v>44.248999999999995</v>
       </c>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A174" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4160,7 +4187,7 @@
         <v>45.839999999999996</v>
       </c>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A175" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4183,7 +4210,7 @@
         <v>47.326999999999998</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A176" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4204,7 +4231,7 @@
         <v>48.997999999999998</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A177" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4225,7 +4252,7 @@
         <v>50.769999999999996</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A178" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4246,7 +4273,7 @@
         <v>52.371999999999993</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A179" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4267,7 +4294,7 @@
         <v>54.019999999999996</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A180" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4288,7 +4315,7 @@
         <v>55.545999999999999</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A181" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4309,7 +4336,7 @@
         <v>57.247</v>
       </c>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A182" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4332,7 +4359,7 @@
         <v>58.192</v>
       </c>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A183" t="str">
         <f t="shared" ref="A183:A189" si="13">"Thomas2007"&amp;C183</f>
         <v>Thomas2007OMD76</v>
@@ -4353,7 +4380,7 @@
         <v>59.49</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A184" t="str">
         <f t="shared" si="13"/>
         <v>Thomas2007OMD76</v>
@@ -4374,7 +4401,7 @@
         <v>60.722000000000001</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A185" t="str">
         <f t="shared" si="13"/>
         <v>Thomas2007OMD76</v>
@@ -4395,7 +4422,7 @@
         <v>62.097000000000001</v>
       </c>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A186" t="str">
         <f t="shared" si="13"/>
         <v>Thomas2007OMD76</v>
@@ -4416,7 +4443,7 @@
         <v>63.569000000000003</v>
       </c>
     </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A187" t="str">
         <f t="shared" si="13"/>
         <v>Thomas2007OMD76</v>
@@ -4437,7 +4464,7 @@
         <v>64.948000000000008</v>
       </c>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A188" t="str">
         <f t="shared" si="13"/>
         <v>Thomas2007OMD76</v>
@@ -4458,7 +4485,7 @@
         <v>66.381000000000014</v>
       </c>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A189" t="str">
         <f t="shared" si="13"/>
         <v>Thomas2007OMD76</v>
@@ -4480,8 +4507,11 @@
         <f t="shared" si="11"/>
         <v>67.715000000000018</v>
       </c>
-    </row>
-    <row r="1048564" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="J189">
+        <v>1.9590000000000001</v>
+      </c>
+    </row>
+    <row r="1048564" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D1048564" s="1"/>
     </row>
   </sheetData>
@@ -4497,9 +4527,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05D3643E-19A9-4BCA-984E-D3604CFC9FB7}">
   <dimension ref="A1:I200"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>13</v>
       </c>
@@ -4528,7 +4558,7 @@
         <v>1315</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>13</v>
       </c>
@@ -4557,7 +4587,7 @@
         <v>1310</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
@@ -4586,7 +4616,7 @@
         <v>1590</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
@@ -4615,7 +4645,7 @@
         <v>1908</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
@@ -4644,7 +4674,7 @@
         <v>1701</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>13</v>
       </c>
@@ -4673,7 +4703,7 @@
         <v>1661</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>13</v>
       </c>
@@ -4702,7 +4732,7 @@
         <v>1753</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>13</v>
       </c>
@@ -4731,7 +4761,7 @@
         <v>1655</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>13</v>
       </c>
@@ -4760,7 +4790,7 @@
         <v>1704</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>13</v>
       </c>
@@ -4789,7 +4819,7 @@
         <v>1529</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>13</v>
       </c>
@@ -4818,7 +4848,7 @@
         <v>1729</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>13</v>
       </c>
@@ -4847,7 +4877,7 @@
         <v>1716</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>13</v>
       </c>
@@ -4876,7 +4906,7 @@
         <v>1549</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>13</v>
       </c>
@@ -4905,7 +4935,7 @@
         <v>1847</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
@@ -4934,7 +4964,7 @@
         <v>1572</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>13</v>
       </c>
@@ -4963,7 +4993,7 @@
         <v>1371</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>13</v>
       </c>
@@ -4992,7 +5022,7 @@
         <v>1531</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>13</v>
       </c>
@@ -5021,7 +5051,7 @@
         <v>1539</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>13</v>
       </c>
@@ -5050,7 +5080,7 @@
         <v>2143</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>13</v>
       </c>
@@ -5079,7 +5109,7 @@
         <v>1738</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>13</v>
       </c>
@@ -5108,7 +5138,7 @@
         <v>1620</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>13</v>
       </c>
@@ -5137,7 +5167,7 @@
         <v>1802</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>13</v>
       </c>
@@ -5166,7 +5196,7 @@
         <v>1710</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>13</v>
       </c>
@@ -5195,7 +5225,7 @@
         <v>1592</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>13</v>
       </c>
@@ -5224,7 +5254,7 @@
         <v>1397</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>13</v>
       </c>
@@ -5253,7 +5283,7 @@
         <v>1333</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>13</v>
       </c>
@@ -5282,7 +5312,7 @@
         <v>1429</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>13</v>
       </c>
@@ -5311,7 +5341,7 @@
         <v>1660</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>13</v>
       </c>
@@ -5340,7 +5370,7 @@
         <v>1419</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>13</v>
       </c>
@@ -5369,7 +5399,7 @@
         <v>1671</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>13</v>
       </c>
@@ -5398,7 +5428,7 @@
         <v>1653</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>13</v>
       </c>
@@ -5427,7 +5457,7 @@
         <v>1711</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>13</v>
       </c>
@@ -5456,7 +5486,7 @@
         <v>1680</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>13</v>
       </c>
@@ -5485,7 +5515,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>13</v>
       </c>
@@ -5514,7 +5544,7 @@
         <v>1516</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>13</v>
       </c>
@@ -5543,7 +5573,7 @@
         <v>1671</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>13</v>
       </c>
@@ -5572,7 +5602,7 @@
         <v>1612</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>13</v>
       </c>
@@ -5601,7 +5631,7 @@
         <v>1532</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>13</v>
       </c>
@@ -5630,7 +5660,7 @@
         <v>1729</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>13</v>
       </c>
@@ -5659,7 +5689,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>13</v>
       </c>
@@ -5688,7 +5718,7 @@
         <v>1170</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>13</v>
       </c>
@@ -5717,7 +5747,7 @@
         <v>1419</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>13</v>
       </c>
@@ -5746,7 +5776,7 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>13</v>
       </c>
@@ -5775,7 +5805,7 @@
         <v>1205</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>13</v>
       </c>
@@ -5804,7 +5834,7 @@
         <v>1232</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>13</v>
       </c>
@@ -5833,7 +5863,7 @@
         <v>1227</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>13</v>
       </c>
@@ -5862,7 +5892,7 @@
         <v>1172</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>14</v>
       </c>
@@ -5875,7 +5905,7 @@
       <c r="H48" s="3"/>
       <c r="I48" s="3"/>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>14</v>
       </c>
@@ -5888,7 +5918,7 @@
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>14</v>
       </c>
@@ -5901,7 +5931,7 @@
       <c r="H50" s="3"/>
       <c r="I50" s="3"/>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>14</v>
       </c>
@@ -5914,7 +5944,7 @@
       <c r="H51" s="3"/>
       <c r="I51" s="3"/>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>14</v>
       </c>
@@ -5943,7 +5973,7 @@
         <v>1911</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>14</v>
       </c>
@@ -5972,7 +6002,7 @@
         <v>1909</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>14</v>
       </c>
@@ -6001,7 +6031,7 @@
         <v>1899</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>14</v>
       </c>
@@ -6030,7 +6060,7 @@
         <v>2003</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>14</v>
       </c>
@@ -6059,7 +6089,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>14</v>
       </c>
@@ -6088,7 +6118,7 @@
         <v>1765</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>14</v>
       </c>
@@ -6117,7 +6147,7 @@
         <v>1953</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>14</v>
       </c>
@@ -6146,7 +6176,7 @@
         <v>1921</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>14</v>
       </c>
@@ -6175,7 +6205,7 @@
         <v>1761</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>14</v>
       </c>
@@ -6204,7 +6234,7 @@
         <v>1894</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
         <v>14</v>
       </c>
@@ -6233,7 +6263,7 @@
         <v>1856</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>14</v>
       </c>
@@ -6262,7 +6292,7 @@
         <v>1719</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>14</v>
       </c>
@@ -6291,7 +6321,7 @@
         <v>1888</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
         <v>14</v>
       </c>
@@ -6320,7 +6350,7 @@
         <v>1907</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
         <v>14</v>
       </c>
@@ -6349,7 +6379,7 @@
         <v>1890</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
         <v>14</v>
       </c>
@@ -6378,7 +6408,7 @@
         <v>1510</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
         <v>14</v>
       </c>
@@ -6407,7 +6437,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>14</v>
       </c>
@@ -6436,7 +6466,7 @@
         <v>1700</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>14</v>
       </c>
@@ -6465,7 +6495,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>14</v>
       </c>
@@ -6494,7 +6524,7 @@
         <v>1731</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
         <v>14</v>
       </c>
@@ -6523,7 +6553,7 @@
         <v>1989</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>14</v>
       </c>
@@ -6552,7 +6582,7 @@
         <v>1896</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>14</v>
       </c>
@@ -6581,7 +6611,7 @@
         <v>1745</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>14</v>
       </c>
@@ -6610,7 +6640,7 @@
         <v>1859</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>14</v>
       </c>
@@ -6639,7 +6669,7 @@
         <v>1949</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>14</v>
       </c>
@@ -6668,7 +6698,7 @@
         <v>1865</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
         <v>14</v>
       </c>
@@ -6697,7 +6727,7 @@
         <v>1920</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
         <v>14</v>
       </c>
@@ -6726,7 +6756,7 @@
         <v>1846</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
         <v>14</v>
       </c>
@@ -6755,7 +6785,7 @@
         <v>1790</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>14</v>
       </c>
@@ -6784,7 +6814,7 @@
         <v>1748</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
         <v>14</v>
       </c>
@@ -6813,7 +6843,7 @@
         <v>1807</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>14</v>
       </c>
@@ -6842,7 +6872,7 @@
         <v>1869</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>14</v>
       </c>
@@ -6871,7 +6901,7 @@
         <v>1696</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>14</v>
       </c>
@@ -6900,7 +6930,7 @@
         <v>2045</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>14</v>
       </c>
@@ -6929,7 +6959,7 @@
         <v>1786</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>14</v>
       </c>
@@ -6958,7 +6988,7 @@
         <v>1865</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
         <v>14</v>
       </c>
@@ -6987,7 +7017,7 @@
         <v>1770</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>14</v>
       </c>
@@ -7016,7 +7046,7 @@
         <v>1772</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>14</v>
       </c>
@@ -7045,7 +7075,7 @@
         <v>1780</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
         <v>14</v>
       </c>
@@ -7074,7 +7104,7 @@
         <v>1296</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
         <v>14</v>
       </c>
@@ -7103,7 +7133,7 @@
         <v>1370</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
         <v>14</v>
       </c>
@@ -7132,7 +7162,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
         <v>14</v>
       </c>
@@ -7161,7 +7191,7 @@
         <v>1078</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
         <v>14</v>
       </c>
@@ -7190,7 +7220,7 @@
         <v>1312</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
         <v>14</v>
       </c>
@@ -7219,7 +7249,7 @@
         <v>1241</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
         <v>14</v>
       </c>
@@ -7248,7 +7278,7 @@
         <v>1249</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
         <v>14</v>
       </c>
@@ -7277,7 +7307,7 @@
         <v>1163</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
         <v>15</v>
       </c>
@@ -7290,7 +7320,7 @@
       <c r="H99" s="3"/>
       <c r="I99" s="3"/>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
         <v>15</v>
       </c>
@@ -7303,7 +7333,7 @@
       <c r="H100" s="3"/>
       <c r="I100" s="3"/>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
         <v>15</v>
       </c>
@@ -7316,7 +7346,7 @@
       <c r="H101" s="3"/>
       <c r="I101" s="3"/>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
         <v>15</v>
       </c>
@@ -7329,7 +7359,7 @@
       <c r="H102" s="3"/>
       <c r="I102" s="3"/>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
         <v>15</v>
       </c>
@@ -7358,7 +7388,7 @@
         <v>2110</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
         <v>15</v>
       </c>
@@ -7387,7 +7417,7 @@
         <v>1863</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
         <v>15</v>
       </c>
@@ -7416,7 +7446,7 @@
         <v>1937</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
         <v>15</v>
       </c>
@@ -7445,7 +7475,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
         <v>15</v>
       </c>
@@ -7474,7 +7504,7 @@
         <v>1981</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
         <v>15</v>
       </c>
@@ -7503,7 +7533,7 @@
         <v>1854</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
         <v>15</v>
       </c>
@@ -7532,7 +7562,7 @@
         <v>1610</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
         <v>15</v>
       </c>
@@ -7561,7 +7591,7 @@
         <v>1911</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="s">
         <v>15</v>
       </c>
@@ -7590,7 +7620,7 @@
         <v>1740</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="3" t="s">
         <v>15</v>
       </c>
@@ -7619,7 +7649,7 @@
         <v>1880</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
         <v>15</v>
       </c>
@@ -7648,7 +7678,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="s">
         <v>15</v>
       </c>
@@ -7677,7 +7707,7 @@
         <v>1859</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="3" t="s">
         <v>15</v>
       </c>
@@ -7706,7 +7736,7 @@
         <v>1870</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" s="3" t="s">
         <v>15</v>
       </c>
@@ -7735,7 +7765,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="3" t="s">
         <v>15</v>
       </c>
@@ -7764,7 +7794,7 @@
         <v>1815</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="s">
         <v>15</v>
       </c>
@@ -7793,7 +7823,7 @@
         <v>1608</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="s">
         <v>15</v>
       </c>
@@ -7822,7 +7852,7 @@
         <v>1797</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
         <v>15</v>
       </c>
@@ -7851,7 +7881,7 @@
         <v>1541</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
         <v>15</v>
       </c>
@@ -7880,7 +7910,7 @@
         <v>1579</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" s="3" t="s">
         <v>15</v>
       </c>
@@ -7909,7 +7939,7 @@
         <v>1533</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" s="3" t="s">
         <v>15</v>
       </c>
@@ -7938,7 +7968,7 @@
         <v>1413</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
         <v>15</v>
       </c>
@@ -7967,7 +7997,7 @@
         <v>1485</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" s="3" t="s">
         <v>15</v>
       </c>
@@ -7996,7 +8026,7 @@
         <v>1509</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
         <v>15</v>
       </c>
@@ -8025,7 +8055,7 @@
         <v>1540</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
         <v>15</v>
       </c>
@@ -8054,7 +8084,7 @@
         <v>1778</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
         <v>15</v>
       </c>
@@ -8083,7 +8113,7 @@
         <v>1651</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="3" t="s">
         <v>15</v>
       </c>
@@ -8112,7 +8142,7 @@
         <v>1751</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" s="3" t="s">
         <v>15</v>
       </c>
@@ -8141,7 +8171,7 @@
         <v>1991</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" s="3" t="s">
         <v>15</v>
       </c>
@@ -8170,7 +8200,7 @@
         <v>1690</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
         <v>15</v>
       </c>
@@ -8199,7 +8229,7 @@
         <v>2127</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" s="3" t="s">
         <v>15</v>
       </c>
@@ -8228,7 +8258,7 @@
         <v>1708</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="3" t="s">
         <v>15</v>
       </c>
@@ -8257,7 +8287,7 @@
         <v>1650</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" s="3" t="s">
         <v>15</v>
       </c>
@@ -8286,7 +8316,7 @@
         <v>1741</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="3" t="s">
         <v>15</v>
       </c>
@@ -8315,7 +8345,7 @@
         <v>1898</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="s">
         <v>15</v>
       </c>
@@ -8344,7 +8374,7 @@
         <v>1694</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" s="3" t="s">
         <v>15</v>
       </c>
@@ -8373,7 +8403,7 @@
         <v>1732</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" s="3" t="s">
         <v>15</v>
       </c>
@@ -8402,7 +8432,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="3" t="s">
         <v>15</v>
       </c>
@@ -8431,7 +8461,7 @@
         <v>1744</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="3" t="s">
         <v>15</v>
       </c>
@@ -8460,7 +8490,7 @@
         <v>1820</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" s="3" t="s">
         <v>15</v>
       </c>
@@ -8489,7 +8519,7 @@
         <v>1085</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" s="3" t="s">
         <v>15</v>
       </c>
@@ -8518,7 +8548,7 @@
         <v>1460</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" s="3" t="s">
         <v>15</v>
       </c>
@@ -8547,7 +8577,7 @@
         <v>1116</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" s="3" t="s">
         <v>15</v>
       </c>
@@ -8576,7 +8606,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" s="3" t="s">
         <v>15</v>
       </c>
@@ -8605,7 +8635,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
         <v>15</v>
       </c>
@@ -8634,7 +8664,7 @@
         <v>1285</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" s="3" t="s">
         <v>15</v>
       </c>
@@ -8663,7 +8693,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" s="3" t="s">
         <v>15</v>
       </c>
@@ -8692,7 +8722,7 @@
         <v>1396</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" s="3" t="s">
         <v>16</v>
       </c>
@@ -8705,7 +8735,7 @@
       <c r="H150" s="3"/>
       <c r="I150" s="3"/>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" s="3" t="s">
         <v>16</v>
       </c>
@@ -8718,7 +8748,7 @@
       <c r="H151" s="3"/>
       <c r="I151" s="3"/>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" s="3" t="s">
         <v>16</v>
       </c>
@@ -8731,7 +8761,7 @@
       <c r="H152" s="3"/>
       <c r="I152" s="3"/>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" s="3" t="s">
         <v>16</v>
       </c>
@@ -8744,7 +8774,7 @@
       <c r="H153" s="3"/>
       <c r="I153" s="3"/>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" s="3" t="s">
         <v>16</v>
       </c>
@@ -8773,7 +8803,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" s="3" t="s">
         <v>16</v>
       </c>
@@ -8802,7 +8832,7 @@
         <v>1553</v>
       </c>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" s="3" t="s">
         <v>16</v>
       </c>
@@ -8831,7 +8861,7 @@
         <v>1746</v>
       </c>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" s="3" t="s">
         <v>16</v>
       </c>
@@ -8860,7 +8890,7 @@
         <v>1677</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" s="3" t="s">
         <v>16</v>
       </c>
@@ -8889,7 +8919,7 @@
         <v>1971</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" s="3" t="s">
         <v>16</v>
       </c>
@@ -8918,7 +8948,7 @@
         <v>1444</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" s="3" t="s">
         <v>16</v>
       </c>
@@ -8947,7 +8977,7 @@
         <v>1884</v>
       </c>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" s="3" t="s">
         <v>16</v>
       </c>
@@ -8976,7 +9006,7 @@
         <v>1840</v>
       </c>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" s="3" t="s">
         <v>16</v>
       </c>
@@ -9005,7 +9035,7 @@
         <v>1871</v>
       </c>
     </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" s="3" t="s">
         <v>16</v>
       </c>
@@ -9034,7 +9064,7 @@
         <v>1716</v>
       </c>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" s="3" t="s">
         <v>16</v>
       </c>
@@ -9063,7 +9093,7 @@
         <v>1844</v>
       </c>
     </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" s="3" t="s">
         <v>16</v>
       </c>
@@ -9092,7 +9122,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" s="3" t="s">
         <v>16</v>
       </c>
@@ -9121,7 +9151,7 @@
         <v>1732</v>
       </c>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" s="3" t="s">
         <v>16</v>
       </c>
@@ -9150,7 +9180,7 @@
         <v>1742</v>
       </c>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" s="3" t="s">
         <v>16</v>
       </c>
@@ -9179,7 +9209,7 @@
         <v>1782</v>
       </c>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A169" s="3" t="s">
         <v>16</v>
       </c>
@@ -9208,7 +9238,7 @@
         <v>1218</v>
       </c>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A170" s="3" t="s">
         <v>16</v>
       </c>
@@ -9237,7 +9267,7 @@
         <v>1644</v>
       </c>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A171" s="3" t="s">
         <v>16</v>
       </c>
@@ -9266,7 +9296,7 @@
         <v>1653</v>
       </c>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172" s="3" t="s">
         <v>16</v>
       </c>
@@ -9295,7 +9325,7 @@
         <v>1506</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" s="3" t="s">
         <v>16</v>
       </c>
@@ -9324,7 +9354,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" s="3" t="s">
         <v>16</v>
       </c>
@@ -9353,7 +9383,7 @@
         <v>1644</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A175" s="3" t="s">
         <v>16</v>
       </c>
@@ -9382,7 +9412,7 @@
         <v>1656</v>
       </c>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A176" s="3" t="s">
         <v>16</v>
       </c>
@@ -9411,7 +9441,7 @@
         <v>1395</v>
       </c>
     </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" s="3" t="s">
         <v>16</v>
       </c>
@@ -9440,7 +9470,7 @@
         <v>1572</v>
       </c>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A178" s="3" t="s">
         <v>16</v>
       </c>
@@ -9469,7 +9499,7 @@
         <v>1707</v>
       </c>
     </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A179" s="3" t="s">
         <v>16</v>
       </c>
@@ -9498,7 +9528,7 @@
         <v>1576</v>
       </c>
     </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A180" s="3" t="s">
         <v>16</v>
       </c>
@@ -9527,7 +9557,7 @@
         <v>1545</v>
       </c>
     </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" s="3" t="s">
         <v>16</v>
       </c>
@@ -9556,7 +9586,7 @@
         <v>1494</v>
       </c>
     </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" s="3" t="s">
         <v>16</v>
       </c>
@@ -9585,7 +9615,7 @@
         <v>1598</v>
       </c>
     </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" s="3" t="s">
         <v>16</v>
       </c>
@@ -9614,7 +9644,7 @@
         <v>1608</v>
       </c>
     </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" s="3" t="s">
         <v>16</v>
       </c>
@@ -9643,7 +9673,7 @@
         <v>1578</v>
       </c>
     </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A185" s="3" t="s">
         <v>16</v>
       </c>
@@ -9672,7 +9702,7 @@
         <v>1591</v>
       </c>
     </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A186" s="3" t="s">
         <v>16</v>
       </c>
@@ -9701,7 +9731,7 @@
         <v>1487</v>
       </c>
     </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" s="3" t="s">
         <v>16</v>
       </c>
@@ -9730,7 +9760,7 @@
         <v>1671</v>
       </c>
     </row>
-    <row r="188" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" s="3" t="s">
         <v>16</v>
       </c>
@@ -9759,7 +9789,7 @@
         <v>1772</v>
       </c>
     </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" s="3" t="s">
         <v>16</v>
       </c>
@@ -9788,7 +9818,7 @@
         <v>1602</v>
       </c>
     </row>
-    <row r="190" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" s="3" t="s">
         <v>16</v>
       </c>
@@ -9817,7 +9847,7 @@
         <v>1648</v>
       </c>
     </row>
-    <row r="191" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A191" s="3" t="s">
         <v>16</v>
       </c>
@@ -9846,7 +9876,7 @@
         <v>1526</v>
       </c>
     </row>
-    <row r="192" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A192" s="3" t="s">
         <v>16</v>
       </c>
@@ -9875,7 +9905,7 @@
         <v>1701</v>
       </c>
     </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A193" s="3" t="s">
         <v>16</v>
       </c>
@@ -9904,7 +9934,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A194" s="3" t="s">
         <v>16</v>
       </c>
@@ -9933,7 +9963,7 @@
         <v>1298</v>
       </c>
     </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A195" s="3" t="s">
         <v>16</v>
       </c>
@@ -9962,7 +9992,7 @@
         <v>1232</v>
       </c>
     </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A196" s="3" t="s">
         <v>16</v>
       </c>
@@ -9991,7 +10021,7 @@
         <v>1375</v>
       </c>
     </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A197" s="3" t="s">
         <v>16</v>
       </c>
@@ -10020,7 +10050,7 @@
         <v>1472</v>
       </c>
     </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A198" s="3" t="s">
         <v>16</v>
       </c>
@@ -10049,7 +10079,7 @@
         <v>1379</v>
       </c>
     </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A199" s="3" t="s">
         <v>16</v>
       </c>
@@ -10078,7 +10108,7 @@
         <v>1433</v>
       </c>
     </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A200" s="3" t="s">
         <v>16</v>
       </c>
@@ -10115,14 +10145,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42555D67-1672-42AA-A340-3C90B34A600E}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -10136,7 +10166,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0</v>
       </c>
@@ -10144,7 +10174,7 @@
         <v>281.10000000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>45</v>
       </c>
@@ -10167,7 +10197,7 @@
         <v>10.600888888888887</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>75</v>
       </c>
@@ -10190,7 +10220,7 @@
         <v>9.4210666666666665</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>105</v>
       </c>

</xml_diff>

<commit_message>
Update Thomas2007 fleece data file and starting value and included new figure
</commit_message>
<xml_diff>
--- a/Tests/Validation/Stock/Thomas2007Observed.xlsx
+++ b/Tests/Validation/Stock/Thomas2007Observed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KEO027\ApsimX\Tests\Validation\Stock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61FEA6B5-4482-4C4A-B4DF-601D2498AB2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D07782B-774D-410F-9145-9911B87A7746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="24">
   <si>
     <t>SimulationName</t>
   </si>
@@ -107,6 +107,9 @@
   </si>
   <si>
     <t>Stock.CFleeceWtAll</t>
+  </si>
+  <si>
+    <t>Stock.CFleeceGrowthAll</t>
   </si>
 </sst>
 </file>
@@ -449,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J1048564"/>
+  <dimension ref="A1:K1048564"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
@@ -463,7 +466,7 @@
     <col min="15" max="15" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -494,8 +497,11 @@
       <c r="J1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f t="shared" ref="A2:A33" si="0">"Thomas2007"&amp;C2</f>
         <v>Thomas2007OMD55</v>
@@ -512,7 +518,7 @@
       </c>
       <c r="G2" s="3"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -530,7 +536,7 @@
       </c>
       <c r="G3" s="3"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -548,7 +554,7 @@
       </c>
       <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -566,7 +572,7 @@
       </c>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -590,7 +596,7 @@
         <v>1.7010000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -612,7 +618,7 @@
         <v>3.3620000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -634,7 +640,7 @@
         <v>5.1150000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -656,7 +662,7 @@
         <v>6.7700000000000005</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -678,7 +684,7 @@
         <v>8.4740000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -700,7 +706,7 @@
         <v>10.003</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -722,7 +728,7 @@
         <v>11.731999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -746,7 +752,7 @@
         <v>13.447999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -768,7 +774,7 @@
         <v>14.996999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -790,7 +796,7 @@
         <v>16.843999999999998</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -812,7 +818,7 @@
         <v>18.415999999999997</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -834,7 +840,7 @@
         <v>19.786999999999995</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -856,7 +862,7 @@
         <v>21.317999999999994</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -878,7 +884,7 @@
         <v>22.856999999999996</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -902,10 +908,13 @@
         <v>24.999999999999996</v>
       </c>
       <c r="J20">
-        <v>1.36</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.69968785791308608</v>
+      </c>
+      <c r="K20">
+        <v>1.7785400126356904E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -927,7 +936,7 @@
         <v>26.737999999999996</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -949,7 +958,7 @@
         <v>28.357999999999997</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -971,7 +980,7 @@
         <v>30.159999999999997</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -993,7 +1002,7 @@
         <v>31.869999999999997</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1015,7 +1024,7 @@
         <v>33.461999999999996</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1037,7 +1046,7 @@
         <v>34.858999999999995</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1061,7 +1070,7 @@
         <v>36.191999999999993</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1083,7 +1092,7 @@
         <v>37.620999999999995</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1105,7 +1114,7 @@
         <v>39.280999999999992</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1127,7 +1136,7 @@
         <v>40.699999999999989</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1149,7 +1158,7 @@
         <v>42.370999999999988</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1171,7 +1180,7 @@
         <v>44.023999999999987</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1193,7 +1202,7 @@
         <v>45.734999999999985</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="str">
         <f t="shared" ref="A34:A65" si="3">"Thomas2007"&amp;C34</f>
         <v>Thomas2007OMD55</v>
@@ -1217,7 +1226,7 @@
         <v>47.414999999999985</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1239,7 +1248,7 @@
         <v>49.031999999999982</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1261,7 +1270,7 @@
         <v>50.547999999999981</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1283,7 +1292,7 @@
         <v>52.21899999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1305,7 +1314,7 @@
         <v>53.830999999999982</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1327,7 +1336,7 @@
         <v>55.362999999999985</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1349,7 +1358,7 @@
         <v>57.091999999999985</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1373,8 +1382,14 @@
         <v>58.247999999999983</v>
       </c>
       <c r="I41" s="2"/>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J41">
+        <v>0.9978542663362342</v>
+      </c>
+      <c r="K41">
+        <v>1.4198400401102292E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1397,7 +1412,7 @@
       </c>
       <c r="I42" s="2"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1420,7 +1435,7 @@
       </c>
       <c r="I43" s="2"/>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1443,7 +1458,7 @@
       </c>
       <c r="I44" s="2"/>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1466,7 +1481,7 @@
       </c>
       <c r="I45" s="2"/>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1489,7 +1504,7 @@
       </c>
       <c r="I46" s="2"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1512,7 +1527,7 @@
       </c>
       <c r="I47" s="2"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD55</v>
@@ -1536,9 +1551,6 @@
         <v>67.006999999999991</v>
       </c>
       <c r="I48" s="2"/>
-      <c r="J48">
-        <v>1.95</v>
-      </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="str">
@@ -1864,7 +1876,7 @@
         <v>21.922000000000004</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1885,7 +1897,7 @@
         <v>23.846000000000004</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="str">
         <f t="shared" ref="A66:A97" si="6">"Thomas2007"&amp;C66</f>
         <v>Thomas2007OMD62</v>
@@ -1906,7 +1918,7 @@
         <v>25.546000000000003</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -1929,10 +1941,13 @@
         <v>27.470000000000002</v>
       </c>
       <c r="J67">
-        <v>1.0589999999999999</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.53480966591716261</v>
+      </c>
+      <c r="K67">
+        <v>1.420663530039396E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -1953,7 +1968,7 @@
         <v>29.201000000000004</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -1974,7 +1989,7 @@
         <v>31.190000000000005</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -1995,7 +2010,7 @@
         <v>33.086000000000006</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2016,7 +2031,7 @@
         <v>34.831000000000003</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2037,7 +2052,7 @@
         <v>36.690000000000005</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2058,7 +2073,7 @@
         <v>38.639000000000003</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2081,7 +2096,7 @@
         <v>40.504000000000005</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2102,7 +2117,7 @@
         <v>42.424000000000007</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2123,7 +2138,7 @@
         <v>44.27000000000001</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2144,7 +2159,7 @@
         <v>46.060000000000009</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2165,7 +2180,7 @@
         <v>47.808000000000007</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2186,7 +2201,7 @@
         <v>49.615000000000009</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2207,7 +2222,7 @@
         <v>51.484000000000009</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2230,7 +2245,7 @@
         <v>53.180000000000007</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2251,7 +2266,7 @@
         <v>55.225000000000009</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2272,7 +2287,7 @@
         <v>57.01100000000001</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2293,7 +2308,7 @@
         <v>58.876000000000012</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2314,7 +2329,7 @@
         <v>60.646000000000015</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2335,7 +2350,7 @@
         <v>62.418000000000013</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2356,7 +2371,7 @@
         <v>64.198000000000008</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2378,8 +2393,14 @@
         <f t="shared" si="4"/>
         <v>65.494000000000014</v>
       </c>
-    </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J88">
+        <v>0.83420084909792858</v>
+      </c>
+      <c r="K88">
+        <v>1.4256723008607903E-2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2400,7 +2421,7 @@
         <v>66.864000000000019</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2421,7 +2442,7 @@
         <v>67.793000000000021</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2442,7 +2463,7 @@
         <v>68.871000000000024</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2463,7 +2484,7 @@
         <v>70.183000000000021</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2484,7 +2505,7 @@
         <v>71.424000000000021</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2505,7 +2526,7 @@
         <v>72.673000000000016</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2527,11 +2548,8 @@
         <f t="shared" si="4"/>
         <v>73.836000000000013</v>
       </c>
-      <c r="J95">
-        <v>1.645</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD69</v>
@@ -2875,7 +2893,7 @@
         <v>23.807000000000002</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2896,7 +2914,7 @@
         <v>25.348000000000003</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2919,10 +2937,13 @@
         <v>26.927000000000003</v>
       </c>
       <c r="J114">
-        <v>1.286</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.67399306346768062</v>
+      </c>
+      <c r="K114">
+        <v>1.7600052298964223E-2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2943,7 +2964,7 @@
         <v>28.460000000000004</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2964,7 +2985,7 @@
         <v>29.873000000000005</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2985,7 +3006,7 @@
         <v>31.358000000000004</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3006,7 +3027,7 @@
         <v>32.867000000000004</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3027,7 +3048,7 @@
         <v>34.407000000000004</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3048,7 +3069,7 @@
         <v>36.185000000000002</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3071,7 +3092,7 @@
         <v>37.836000000000006</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3092,7 +3113,7 @@
         <v>39.587000000000003</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3113,7 +3134,7 @@
         <v>41.578000000000003</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3134,7 +3155,7 @@
         <v>43.268000000000001</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3155,7 +3176,7 @@
         <v>45.395000000000003</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3176,7 +3197,7 @@
         <v>47.103000000000002</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3197,7 +3218,7 @@
         <v>48.753</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3220,7 +3241,7 @@
         <v>50.494</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A129" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3241,7 +3262,7 @@
         <v>52.392000000000003</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A130" t="str">
         <f t="shared" ref="A130:A161" si="10">"Thomas2007"&amp;C130</f>
         <v>Thomas2007OMD69</v>
@@ -3262,7 +3283,7 @@
         <v>54.086000000000006</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A131" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3283,7 +3304,7 @@
         <v>55.818000000000005</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A132" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3304,7 +3325,7 @@
         <v>57.465000000000003</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A133" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3325,7 +3346,7 @@
         <v>59.209000000000003</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A134" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3346,7 +3367,7 @@
         <v>61.029000000000003</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A135" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3368,8 +3389,14 @@
         <f t="shared" si="8"/>
         <v>62.114000000000004</v>
       </c>
-    </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J135">
+        <v>1.0328285506409614</v>
+      </c>
+      <c r="K135">
+        <v>1.7087404151108605E-2</v>
+      </c>
+    </row>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A136" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3390,7 +3417,7 @@
         <v>63.574000000000005</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A137" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3411,7 +3438,7 @@
         <v>64.690000000000012</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A138" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3432,7 +3459,7 @@
         <v>65.849000000000018</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A139" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3453,7 +3480,7 @@
         <v>66.982000000000014</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A140" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3474,7 +3501,7 @@
         <v>68.26700000000001</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A141" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3495,7 +3522,7 @@
         <v>69.572000000000017</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A142" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD69</v>
@@ -3517,11 +3544,8 @@
         <f t="shared" si="8"/>
         <v>70.968000000000018</v>
       </c>
-      <c r="J142">
-        <v>1.978</v>
-      </c>
-    </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A143" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3537,7 +3561,7 @@
       </c>
       <c r="G143" s="4"/>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A144" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3886,7 +3910,7 @@
         <v>23.977999999999994</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A161" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3909,10 +3933,13 @@
         <v>25.483999999999995</v>
       </c>
       <c r="J161">
-        <v>1.28</v>
-      </c>
-    </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.63642254540008492</v>
+      </c>
+      <c r="K161">
+        <v>1.6825581080435702E-2</v>
+      </c>
+    </row>
+    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162" t="str">
         <f t="shared" ref="A162:A182" si="12">"Thomas2007"&amp;C162</f>
         <v>Thomas2007OMD76</v>
@@ -3933,7 +3960,7 @@
         <v>26.875999999999994</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A163" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -3954,7 +3981,7 @@
         <v>28.519999999999992</v>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A164" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -3975,7 +4002,7 @@
         <v>30.175999999999991</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A165" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -3996,7 +4023,7 @@
         <v>31.570999999999991</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A166" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4017,7 +4044,7 @@
         <v>33.142999999999994</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A167" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4038,7 +4065,7 @@
         <v>34.849999999999994</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A168" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4061,7 +4088,7 @@
         <v>36.425999999999995</v>
       </c>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A169" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4082,7 +4109,7 @@
         <v>37.970999999999997</v>
       </c>
     </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A170" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4103,7 +4130,7 @@
         <v>39.464999999999996</v>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A171" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4124,7 +4151,7 @@
         <v>41.062999999999995</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A172" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4145,7 +4172,7 @@
         <v>42.670999999999992</v>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A173" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4166,7 +4193,7 @@
         <v>44.248999999999995</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A174" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4187,7 +4214,7 @@
         <v>45.839999999999996</v>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A175" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4210,7 +4237,7 @@
         <v>47.326999999999998</v>
       </c>
     </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A176" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4231,7 +4258,7 @@
         <v>48.997999999999998</v>
       </c>
     </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A177" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4252,7 +4279,7 @@
         <v>50.769999999999996</v>
       </c>
     </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A178" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4273,7 +4300,7 @@
         <v>52.371999999999993</v>
       </c>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A179" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4294,7 +4321,7 @@
         <v>54.019999999999996</v>
       </c>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A180" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4315,7 +4342,7 @@
         <v>55.545999999999999</v>
       </c>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A181" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4336,7 +4363,7 @@
         <v>57.247</v>
       </c>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A182" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4358,8 +4385,14 @@
         <f t="shared" si="11"/>
         <v>58.192</v>
       </c>
-    </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J182">
+        <v>0.9644430836057849</v>
+      </c>
+      <c r="K182">
+        <v>1.5620025628842857E-2</v>
+      </c>
+    </row>
+    <row r="183" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A183" t="str">
         <f t="shared" ref="A183:A189" si="13">"Thomas2007"&amp;C183</f>
         <v>Thomas2007OMD76</v>
@@ -4380,7 +4413,7 @@
         <v>59.49</v>
       </c>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A184" t="str">
         <f t="shared" si="13"/>
         <v>Thomas2007OMD76</v>
@@ -4401,7 +4434,7 @@
         <v>60.722000000000001</v>
       </c>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A185" t="str">
         <f t="shared" si="13"/>
         <v>Thomas2007OMD76</v>
@@ -4422,7 +4455,7 @@
         <v>62.097000000000001</v>
       </c>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A186" t="str">
         <f t="shared" si="13"/>
         <v>Thomas2007OMD76</v>
@@ -4443,7 +4476,7 @@
         <v>63.569000000000003</v>
       </c>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A187" t="str">
         <f t="shared" si="13"/>
         <v>Thomas2007OMD76</v>
@@ -4464,7 +4497,7 @@
         <v>64.948000000000008</v>
       </c>
     </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A188" t="str">
         <f t="shared" si="13"/>
         <v>Thomas2007OMD76</v>
@@ -4485,7 +4518,7 @@
         <v>66.381000000000014</v>
       </c>
     </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A189" t="str">
         <f t="shared" si="13"/>
         <v>Thomas2007OMD76</v>
@@ -4506,9 +4539,6 @@
       <c r="H189">
         <f t="shared" si="11"/>
         <v>67.715000000000018</v>
-      </c>
-      <c r="J189">
-        <v>1.9590000000000001</v>
       </c>
     </row>
     <row r="1048564" spans="4:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated Thomas2007 diet quality and removed initial observed clean fleece weight due to lag effect. Removed basic supplement sensitivity testing
</commit_message>
<xml_diff>
--- a/Tests/Validation/Stock/Thomas2007Observed.xlsx
+++ b/Tests/Validation/Stock/Thomas2007Observed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KEO027\ApsimX\Tests\Validation\Stock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D07782B-774D-410F-9145-9911B87A7746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97AEEDC5-9B58-4D4F-9F62-75A2C35446F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -751,6 +751,10 @@
         <f t="shared" si="2"/>
         <v>13.447999999999999</v>
       </c>
+      <c r="I13">
+        <f>(G13-G6)</f>
+        <v>1.2999999999999972</v>
+      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
@@ -818,7 +822,7 @@
         <v>18.415999999999997</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -840,7 +844,7 @@
         <v>19.786999999999995</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -862,7 +866,7 @@
         <v>21.317999999999994</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -884,7 +888,7 @@
         <v>22.856999999999996</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -907,14 +911,15 @@
         <f t="shared" si="2"/>
         <v>24.999999999999996</v>
       </c>
+      <c r="I20">
+        <f>(G20-G13)+I13</f>
+        <v>0.39999999999999858</v>
+      </c>
       <c r="J20">
         <v>0.69968785791308608</v>
       </c>
-      <c r="K20">
-        <v>1.7785400126356904E-2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -936,7 +941,7 @@
         <v>26.737999999999996</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -958,7 +963,7 @@
         <v>28.357999999999997</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -980,7 +985,7 @@
         <v>30.159999999999997</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1002,7 +1007,7 @@
         <v>31.869999999999997</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1024,7 +1029,7 @@
         <v>33.461999999999996</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1046,7 +1051,7 @@
         <v>34.858999999999995</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1069,8 +1074,12 @@
         <f t="shared" si="2"/>
         <v>36.191999999999993</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I27">
+        <f>(G27-G20)+I20</f>
+        <v>1.8999999999999986</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1092,7 +1101,7 @@
         <v>37.620999999999995</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1114,7 +1123,7 @@
         <v>39.280999999999992</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1136,7 +1145,7 @@
         <v>40.699999999999989</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1158,7 +1167,7 @@
         <v>42.370999999999988</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
         <f t="shared" si="0"/>
         <v>Thomas2007OMD55</v>
@@ -1225,6 +1234,10 @@
         <f t="shared" si="2"/>
         <v>47.414999999999985</v>
       </c>
+      <c r="I34">
+        <f>(G34-G27)+I27</f>
+        <v>1.6999999999999957</v>
+      </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
@@ -1381,7 +1394,10 @@
         <f t="shared" si="2"/>
         <v>58.247999999999983</v>
       </c>
-      <c r="I41" s="2"/>
+      <c r="I41">
+        <f>(G41-G34)+I34</f>
+        <v>2.1000000000000014</v>
+      </c>
       <c r="J41">
         <v>0.9978542663362342</v>
       </c>
@@ -1550,9 +1566,12 @@
         <f t="shared" si="2"/>
         <v>67.006999999999991</v>
       </c>
-      <c r="I48" s="2"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I48">
+        <f>(G48-G41)+I41</f>
+        <v>0.79999999999999716</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1569,7 +1588,7 @@
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1586,7 +1605,7 @@
       </c>
       <c r="G50" s="3"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1603,7 +1622,7 @@
       </c>
       <c r="G51" s="3"/>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1620,7 +1639,7 @@
       </c>
       <c r="G52" s="3"/>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1643,7 +1662,7 @@
         <v>1.8580000000000001</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1664,7 +1683,7 @@
         <v>3.6230000000000002</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1685,7 +1704,7 @@
         <v>5.5760000000000005</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1706,7 +1725,7 @@
         <v>7.4970000000000008</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1727,7 +1746,7 @@
         <v>9.2580000000000009</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1748,7 +1767,7 @@
         <v>11.152000000000001</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1769,7 +1788,7 @@
         <v>13.008000000000001</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1791,8 +1810,12 @@
         <f t="shared" si="4"/>
         <v>14.727</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I60">
+        <f>(G60-G53)</f>
+        <v>0.80000000000000426</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1813,7 +1836,7 @@
         <v>16.615000000000002</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1834,7 +1857,7 @@
         <v>18.522000000000002</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1855,7 +1878,7 @@
         <v>20.412000000000003</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1876,7 +1899,7 @@
         <v>21.922000000000004</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="str">
         <f t="shared" si="3"/>
         <v>Thomas2007OMD62</v>
@@ -1897,7 +1920,7 @@
         <v>23.846000000000004</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="str">
         <f t="shared" ref="A66:A97" si="6">"Thomas2007"&amp;C66</f>
         <v>Thomas2007OMD62</v>
@@ -1918,7 +1941,7 @@
         <v>25.546000000000003</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -1940,14 +1963,15 @@
         <f t="shared" si="4"/>
         <v>27.470000000000002</v>
       </c>
+      <c r="I67">
+        <f>(G67-G60)+I60</f>
+        <v>1.5</v>
+      </c>
       <c r="J67">
         <v>0.53480966591716261</v>
       </c>
-      <c r="K67">
-        <v>1.420663530039396E-2</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -1968,7 +1992,7 @@
         <v>29.201000000000004</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -1989,7 +2013,7 @@
         <v>31.190000000000005</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2010,7 +2034,7 @@
         <v>33.086000000000006</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2031,7 +2055,7 @@
         <v>34.831000000000003</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2052,7 +2076,7 @@
         <v>36.690000000000005</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2073,7 +2097,7 @@
         <v>38.639000000000003</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2095,8 +2119,12 @@
         <f t="shared" si="4"/>
         <v>40.504000000000005</v>
       </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I74">
+        <f>(G74-G67)+I67</f>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2117,7 +2145,7 @@
         <v>42.424000000000007</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2138,7 +2166,7 @@
         <v>44.27000000000001</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2159,7 +2187,7 @@
         <v>46.060000000000009</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2180,7 +2208,7 @@
         <v>47.808000000000007</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2201,7 +2229,7 @@
         <v>49.615000000000009</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD62</v>
@@ -2244,6 +2272,10 @@
         <f t="shared" si="4"/>
         <v>53.180000000000007</v>
       </c>
+      <c r="I81">
+        <f>(G81-G74)+I74</f>
+        <v>3.2000000000000028</v>
+      </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="str">
@@ -2393,6 +2425,10 @@
         <f t="shared" si="4"/>
         <v>65.494000000000014</v>
       </c>
+      <c r="I88">
+        <f>(G88-G81)+I81</f>
+        <v>4.3000000000000043</v>
+      </c>
       <c r="J88">
         <v>0.83420084909792858</v>
       </c>
@@ -2420,6 +2456,7 @@
         <f t="shared" si="4"/>
         <v>66.864000000000019</v>
       </c>
+      <c r="I89" s="2"/>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" t="str">
@@ -2441,6 +2478,7 @@
         <f t="shared" si="4"/>
         <v>67.793000000000021</v>
       </c>
+      <c r="I90" s="2"/>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" t="str">
@@ -2462,6 +2500,7 @@
         <f t="shared" si="4"/>
         <v>68.871000000000024</v>
       </c>
+      <c r="I91" s="2"/>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" t="str">
@@ -2483,6 +2522,7 @@
         <f t="shared" si="4"/>
         <v>70.183000000000021</v>
       </c>
+      <c r="I92" s="2"/>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" t="str">
@@ -2504,6 +2544,7 @@
         <f t="shared" si="4"/>
         <v>71.424000000000021</v>
       </c>
+      <c r="I93" s="2"/>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" t="str">
@@ -2525,6 +2566,7 @@
         <f t="shared" si="4"/>
         <v>72.673000000000016</v>
       </c>
+      <c r="I94" s="2"/>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" t="str">
@@ -2548,6 +2590,10 @@
         <f t="shared" si="4"/>
         <v>73.836000000000013</v>
       </c>
+      <c r="I95">
+        <f>(G95-G88)+I88</f>
+        <v>-1.0999999999999943</v>
+      </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" t="str">
@@ -2565,7 +2611,7 @@
       </c>
       <c r="G96" s="4"/>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" t="str">
         <f t="shared" si="6"/>
         <v>Thomas2007OMD69</v>
@@ -2582,7 +2628,7 @@
       </c>
       <c r="G97" s="3"/>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="str">
         <f t="shared" ref="A98:A129" si="7">"Thomas2007"&amp;C98</f>
         <v>Thomas2007OMD69</v>
@@ -2599,7 +2645,7 @@
       </c>
       <c r="G98" s="3"/>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2616,7 +2662,7 @@
       </c>
       <c r="G99" s="3"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2639,7 +2685,7 @@
         <v>1.9810000000000001</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2660,7 +2706,7 @@
         <v>3.835</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2681,7 +2727,7 @@
         <v>5.4450000000000003</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2702,7 +2748,7 @@
         <v>7.3559999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2723,7 +2769,7 @@
         <v>9.0960000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2744,7 +2790,7 @@
         <v>10.975999999999999</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2765,7 +2811,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2787,8 +2833,12 @@
         <f t="shared" si="8"/>
         <v>14.859</v>
       </c>
-    </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I107">
+        <f>(G107-G100)</f>
+        <v>0.79999999999999716</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2809,7 +2859,7 @@
         <v>16.728999999999999</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2830,7 +2880,7 @@
         <v>18.587</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2851,7 +2901,7 @@
         <v>20.402000000000001</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2872,7 +2922,7 @@
         <v>22.01</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2893,7 +2943,7 @@
         <v>23.807000000000002</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2914,7 +2964,7 @@
         <v>25.348000000000003</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2936,14 +2986,15 @@
         <f t="shared" si="8"/>
         <v>26.927000000000003</v>
       </c>
+      <c r="I114">
+        <f>(G114-G107)+I107</f>
+        <v>1.1999999999999957</v>
+      </c>
       <c r="J114">
         <v>0.67399306346768062</v>
       </c>
-      <c r="K114">
-        <v>1.7600052298964223E-2</v>
-      </c>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2964,7 +3015,7 @@
         <v>28.460000000000004</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -2985,7 +3036,7 @@
         <v>29.873000000000005</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3006,7 +3057,7 @@
         <v>31.358000000000004</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3027,7 +3078,7 @@
         <v>32.867000000000004</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3048,7 +3099,7 @@
         <v>34.407000000000004</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3069,7 +3120,7 @@
         <v>36.185000000000002</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3091,8 +3142,12 @@
         <f t="shared" si="8"/>
         <v>37.836000000000006</v>
       </c>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I121">
+        <f>(G121-G114)+I114</f>
+        <v>1.7999999999999972</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A122" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3113,7 +3168,7 @@
         <v>39.587000000000003</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3134,7 +3189,7 @@
         <v>41.578000000000003</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3155,7 +3210,7 @@
         <v>43.268000000000001</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A125" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3176,7 +3231,7 @@
         <v>45.395000000000003</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A126" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3197,7 +3252,7 @@
         <v>47.103000000000002</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A127" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3218,7 +3273,7 @@
         <v>48.753</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128" t="str">
         <f t="shared" si="7"/>
         <v>Thomas2007OMD69</v>
@@ -3239,6 +3294,10 @@
       <c r="H128">
         <f t="shared" si="8"/>
         <v>50.494</v>
+      </c>
+      <c r="I128">
+        <f>(G128-G121)+I121</f>
+        <v>3.5</v>
       </c>
     </row>
     <row r="129" spans="1:11" x14ac:dyDescent="0.25">
@@ -3389,6 +3448,10 @@
         <f t="shared" si="8"/>
         <v>62.114000000000004</v>
       </c>
+      <c r="I135">
+        <f>(G135-G128)+I128</f>
+        <v>5.3999999999999986</v>
+      </c>
       <c r="J135">
         <v>1.0328285506409614</v>
       </c>
@@ -3416,6 +3479,7 @@
         <f t="shared" si="8"/>
         <v>63.574000000000005</v>
       </c>
+      <c r="I136" s="2"/>
     </row>
     <row r="137" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A137" t="str">
@@ -3437,6 +3501,7 @@
         <f t="shared" si="8"/>
         <v>64.690000000000012</v>
       </c>
+      <c r="I137" s="2"/>
     </row>
     <row r="138" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A138" t="str">
@@ -3458,6 +3523,7 @@
         <f t="shared" si="8"/>
         <v>65.849000000000018</v>
       </c>
+      <c r="I138" s="2"/>
     </row>
     <row r="139" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A139" t="str">
@@ -3479,6 +3545,7 @@
         <f t="shared" si="8"/>
         <v>66.982000000000014</v>
       </c>
+      <c r="I139" s="2"/>
     </row>
     <row r="140" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A140" t="str">
@@ -3500,6 +3567,7 @@
         <f t="shared" si="8"/>
         <v>68.26700000000001</v>
       </c>
+      <c r="I140" s="2"/>
     </row>
     <row r="141" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A141" t="str">
@@ -3521,6 +3589,7 @@
         <f t="shared" si="8"/>
         <v>69.572000000000017</v>
       </c>
+      <c r="I141" s="2"/>
     </row>
     <row r="142" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A142" t="str">
@@ -3544,6 +3613,10 @@
         <f t="shared" si="8"/>
         <v>70.968000000000018</v>
       </c>
+      <c r="I142">
+        <f>(G142-G135)+I135</f>
+        <v>2.2999999999999972</v>
+      </c>
     </row>
     <row r="143" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A143" t="str">
@@ -3578,7 +3651,7 @@
       </c>
       <c r="G144" s="3"/>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3595,7 +3668,7 @@
       </c>
       <c r="G145" s="3"/>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3612,7 +3685,7 @@
       </c>
       <c r="G146" s="3"/>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3635,7 +3708,7 @@
         <v>1.9710000000000001</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3656,7 +3729,7 @@
         <v>3.415</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3677,7 +3750,7 @@
         <v>5.2989999999999995</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3698,7 +3771,7 @@
         <v>7.1389999999999993</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3719,7 +3792,7 @@
         <v>9.01</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3740,7 +3813,7 @@
         <v>10.725999999999999</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3761,7 +3834,7 @@
         <v>12.569999999999999</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3783,8 +3856,12 @@
         <f t="shared" si="11"/>
         <v>14.206999999999999</v>
       </c>
-    </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I154">
+        <f>(G154-G147)</f>
+        <v>1.2000000000000028</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3805,7 +3882,7 @@
         <v>15.938999999999998</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3826,7 +3903,7 @@
         <v>17.680999999999997</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3847,7 +3924,7 @@
         <v>19.462999999999997</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3868,7 +3945,7 @@
         <v>20.680999999999997</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3889,7 +3966,7 @@
         <v>22.324999999999996</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3910,7 +3987,7 @@
         <v>23.977999999999994</v>
       </c>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A161" t="str">
         <f t="shared" si="10"/>
         <v>Thomas2007OMD76</v>
@@ -3932,14 +4009,15 @@
         <f t="shared" si="11"/>
         <v>25.483999999999995</v>
       </c>
+      <c r="I161">
+        <f>(G161-G154)+I154</f>
+        <v>1.5</v>
+      </c>
       <c r="J161">
         <v>0.63642254540008492</v>
       </c>
-      <c r="K161">
-        <v>1.6825581080435702E-2</v>
-      </c>
-    </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A162" t="str">
         <f t="shared" ref="A162:A182" si="12">"Thomas2007"&amp;C162</f>
         <v>Thomas2007OMD76</v>
@@ -3960,7 +4038,7 @@
         <v>26.875999999999994</v>
       </c>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A163" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -3981,7 +4059,7 @@
         <v>28.519999999999992</v>
       </c>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A164" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4002,7 +4080,7 @@
         <v>30.175999999999991</v>
       </c>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A165" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4023,7 +4101,7 @@
         <v>31.570999999999991</v>
       </c>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A166" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4044,7 +4122,7 @@
         <v>33.142999999999994</v>
       </c>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A167" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4065,7 +4143,7 @@
         <v>34.849999999999994</v>
       </c>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A168" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4087,8 +4165,12 @@
         <f t="shared" si="11"/>
         <v>36.425999999999995</v>
       </c>
-    </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I168">
+        <f>(G168-G161)+I161</f>
+        <v>2.2000000000000028</v>
+      </c>
+    </row>
+    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A169" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4109,7 +4191,7 @@
         <v>37.970999999999997</v>
       </c>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A170" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4130,7 +4212,7 @@
         <v>39.464999999999996</v>
       </c>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A171" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4151,7 +4233,7 @@
         <v>41.062999999999995</v>
       </c>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A172" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4172,7 +4254,7 @@
         <v>42.670999999999992</v>
       </c>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A173" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4193,7 +4275,7 @@
         <v>44.248999999999995</v>
       </c>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A174" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4214,7 +4296,7 @@
         <v>45.839999999999996</v>
       </c>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A175" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4236,8 +4318,12 @@
         <f t="shared" si="11"/>
         <v>47.326999999999998</v>
       </c>
-    </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I175">
+        <f>(G175-G168)+I168</f>
+        <v>3.2999999999999972</v>
+      </c>
+    </row>
+    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A176" t="str">
         <f t="shared" si="12"/>
         <v>Thomas2007OMD76</v>
@@ -4385,6 +4471,10 @@
         <f t="shared" si="11"/>
         <v>58.192</v>
       </c>
+      <c r="I182">
+        <f>(G182-G175)+I175</f>
+        <v>5.3999999999999986</v>
+      </c>
       <c r="J182">
         <v>0.9644430836057849</v>
       </c>
@@ -4412,6 +4502,7 @@
         <f t="shared" si="11"/>
         <v>59.49</v>
       </c>
+      <c r="I183" s="2"/>
     </row>
     <row r="184" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A184" t="str">
@@ -4433,6 +4524,7 @@
         <f t="shared" si="11"/>
         <v>60.722000000000001</v>
       </c>
+      <c r="I184" s="2"/>
     </row>
     <row r="185" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A185" t="str">
@@ -4454,6 +4546,7 @@
         <f t="shared" si="11"/>
         <v>62.097000000000001</v>
       </c>
+      <c r="I185" s="2"/>
     </row>
     <row r="186" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A186" t="str">
@@ -4475,6 +4568,7 @@
         <f t="shared" si="11"/>
         <v>63.569000000000003</v>
       </c>
+      <c r="I186" s="2"/>
     </row>
     <row r="187" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A187" t="str">
@@ -4496,6 +4590,7 @@
         <f t="shared" si="11"/>
         <v>64.948000000000008</v>
       </c>
+      <c r="I187" s="2"/>
     </row>
     <row r="188" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A188" t="str">
@@ -4517,6 +4612,7 @@
         <f t="shared" si="11"/>
         <v>66.381000000000014</v>
       </c>
+      <c r="I188" s="2"/>
     </row>
     <row r="189" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A189" t="str">
@@ -4539,6 +4635,10 @@
       <c r="H189">
         <f t="shared" si="11"/>
         <v>67.715000000000018</v>
+      </c>
+      <c r="I189">
+        <f>(G189-G182)+I182</f>
+        <v>2.5</v>
       </c>
     </row>
     <row r="1048564" spans="4:4" x14ac:dyDescent="0.25">

</xml_diff>